<commit_message>
Edit serial 1 Hz in Continuous mode
</commit_message>
<xml_diff>
--- a/measurements/continuous_measurement_20260807_094536.xlsx
+++ b/measurements/continuous_measurement_20260807_094536.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\T.North Job\Rubber tester\Dev v3\Code\oil_project_5_rejectspikeDisplayMega2560_ContinuousIQR_serial\measurements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067E1CB0-EDF9-4CDC-9D14-C30853682C60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE158E3-A03F-431C-A7DC-BF6FAB10E8D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -55,8 +55,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="188" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
-    <numFmt numFmtId="189" formatCode="0.000"/>
+    <numFmt numFmtId="187" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="188" formatCode="0.000"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -106,11 +106,11 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="188" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="187" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="189" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="188" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="ปกติ" xfId="0" builtinId="0"/>
@@ -1020,7 +1020,6 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="t"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -1128,7 +1127,7 @@
           <a:effectLst/>
         </c:spPr>
         <c:txPr>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="0"/>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="0"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
@@ -1496,6 +1495,22 @@
             <c:dispRSqr val="0"/>
             <c:dispEq val="0"/>
           </c:trendline>
+          <c:trendline>
+            <c:name>VMAG Trendline</c:name>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="6"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
           <c:cat>
             <c:numRef>
               <c:f>Data!$A$6:$A$125</c:f>
@@ -2417,7 +2432,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-US"/>
-                  <a:t>VPHS (Vlot)</a:t>
+                  <a:t>VMAG (Vlot)</a:t>
                 </a:r>
                 <a:endParaRPr lang="th-TH"/>
               </a:p>
@@ -2497,6 +2512,10 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
+      <c:legendEntry>
+        <c:idx val="1"/>
+        <c:delete val="1"/>
+      </c:legendEntry>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>

</xml_diff>